<commit_message>
feat: agregar validaciones de redondeo, inicio de campo y caracteres especiales
</commit_message>
<xml_diff>
--- a/Prevalidador/2. archivos/Tapa OPS .xlsx
+++ b/Prevalidador/2. archivos/Tapa OPS .xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://indra365-my.sharepoint.com/personal/dacanonm_indracompany_com/Documents/Documentos/GitHub/automatizacion OPS/Prevalidador/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://indra365-my.sharepoint.com/personal/dacanonm_indracompany_com/Documents/Documentos/GitHub/automatizacion OPS/Prevalidador/2. archivos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{9740106F-1614-4473-B123-A727AECFF786}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6F476DF8-4A98-44B1-9757-FDD101FDAC52}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{9740106F-1614-4473-B123-A727AECFF786}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A3DD9167-2403-4E49-B4BA-D36829BF7CA9}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -560,6 +560,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -882,7 +886,7 @@
     <row r="4" spans="3:16" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="C4" s="26">
         <f ca="1">TODAY()</f>
-        <v>46069</v>
+        <v>46098</v>
       </c>
       <c r="D4" s="27"/>
       <c r="E4" s="27"/>

</xml_diff>